<commit_message>
Update excel and constants
</commit_message>
<xml_diff>
--- a/data/May/Data.xlsx
+++ b/data/May/Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DBC2162-F914-4D85-BC78-3B43D072F096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D1725FD-408C-4A72-9502-2DE738FD0946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="437">
   <si>
     <t>THU 6</t>
   </si>
@@ -940,24 +940,6 @@
     <t>HD018213</t>
   </si>
   <si>
-    <t>27 nguyễn hữu thọ ( sunrise city toà X1)</t>
-  </si>
-  <si>
-    <t>7hcm</t>
-  </si>
-  <si>
-    <t>Hiểu Mỹ</t>
-  </si>
-  <si>
-    <t>HD017734</t>
-  </si>
-  <si>
-    <t>Toà 2, chung cư river panorama, 20 lê thị chợ</t>
-  </si>
-  <si>
-    <t>7don giaslt.tiendon giaao ren pha tua rua</t>
-  </si>
-  <si>
     <t>Trần Thục Oanh</t>
   </si>
   <si>
@@ -970,39 +952,24 @@
     <t>10</t>
   </si>
   <si>
-    <t>Nhưng Bùi</t>
-  </si>
-  <si>
     <t>H0018373</t>
   </si>
   <si>
-    <t>409/108/32/14c huynh thị hai, tán chánh hiệp 2</t>
-  </si>
-  <si>
     <t>Trần Ngọc Thúy</t>
   </si>
   <si>
     <t>HD018516</t>
   </si>
   <si>
-    <t>saigon mia block b cổng sau binh chanh</t>
-  </si>
-  <si>
     <t>Ngọc Vinh</t>
   </si>
   <si>
     <t>HD018285</t>
   </si>
   <si>
-    <t>17-19 Trường Sơn DA</t>
-  </si>
-  <si>
     <t>C. Phương fb Nuory Le</t>
   </si>
   <si>
-    <t>A28/1Dw3 quốc lộ 50 ấp 1 xá lành từng huyện Hình Chính</t>
-  </si>
-  <si>
     <t>ny nhỏ</t>
   </si>
   <si>
@@ -1060,9 +1027,6 @@
     <t>HD018552</t>
   </si>
   <si>
-    <t>Tuyệt Nhi</t>
-  </si>
-  <si>
     <t>HD018231</t>
   </si>
   <si>
@@ -1102,18 +1066,12 @@
     <t>HD018325</t>
   </si>
   <si>
-    <t>56/41 dương ba trạc, Phường 02 , Hồ Chí Minh, Vietnam</t>
-  </si>
-  <si>
     <t>HD018386</t>
   </si>
   <si>
     <t>hàng của Đào Ngọc Bích</t>
   </si>
   <si>
-    <t>007 Lộ B chung cư Tây Thạnh, phương Tần Thạnh, q</t>
-  </si>
-  <si>
     <t>Việt Anh - fb Hồ Thị Uyên</t>
   </si>
   <si>
@@ -1126,9 +1084,6 @@
     <t>HD018494</t>
   </si>
   <si>
-    <t>chung cư the park residence, 12 nguyễn hữu thọ phước kien nha be, D</t>
-  </si>
-  <si>
     <t>cô dung fb Nini Thach</t>
   </si>
   <si>
@@ -1153,9 +1108,6 @@
     <t>HD018437</t>
   </si>
   <si>
-    <t>536/32/23 âu cơ Tân binh</t>
-  </si>
-  <si>
     <t>CN</t>
   </si>
   <si>
@@ -1174,42 +1126,24 @@
     <t>HD017772</t>
   </si>
   <si>
-    <t>290 an dương vương</t>
-  </si>
-  <si>
-    <t>Thao Nguyen Yen chau</t>
-  </si>
-  <si>
     <t>HD018526</t>
   </si>
   <si>
-    <t>Chung cu Horita, lo C, Đường D4, P</t>
-  </si>
-  <si>
     <t>Thư Ánh Võ</t>
   </si>
   <si>
     <t>HD018343</t>
   </si>
   <si>
-    <t>5/te thanh tôn bên nghệ c1</t>
-  </si>
-  <si>
     <t>Châu Châu</t>
   </si>
   <si>
     <t>HD018490</t>
   </si>
   <si>
-    <t>E3/8 ấp 56 xã vĩnh lộc thành phố</t>
-  </si>
-  <si>
     <t>Ly Sokny- 012776599</t>
   </si>
   <si>
-    <t>HD018249</t>
-  </si>
-  <si>
     <t>359 phạm ngũ lão</t>
   </si>
   <si>
@@ -1219,9 +1153,6 @@
     <t>HD018429</t>
   </si>
   <si>
-    <t>30/18 đường số 6 KP18</t>
-  </si>
-  <si>
     <t>Hồng Miên</t>
   </si>
   <si>
@@ -1249,30 +1180,18 @@
     <t>395 Bùi Đình Tuý, p14</t>
   </si>
   <si>
-    <t>Khách tr</t>
-  </si>
-  <si>
     <t>HD018565</t>
   </si>
   <si>
-    <t>171/43 Liên Khu 5-6</t>
-  </si>
-  <si>
     <t>Ivy Dao</t>
   </si>
   <si>
     <t>HD018318</t>
   </si>
   <si>
-    <t>238/3 trường chinh, động hưng thuận .</t>
-  </si>
-  <si>
     <t>HD018376</t>
   </si>
   <si>
-    <t>Loan Thổ</t>
-  </si>
-  <si>
     <t>HD018544</t>
   </si>
   <si>
@@ -1285,9 +1204,6 @@
     <t>HD018549</t>
   </si>
   <si>
-    <t>192 Phạm Đức Sơn, Phường 16 (Chung Cư Heaven Riverview</t>
-  </si>
-  <si>
     <t>Mỹ Ngọc</t>
   </si>
   <si>
@@ -1297,27 +1213,12 @@
     <t>Nguyễn Minh Hải</t>
   </si>
   <si>
-    <t>17 Dương Số 13 Bình Hưng Hoà Bình Tân Tp</t>
-  </si>
-  <si>
-    <t>Nguyễn Minh Hai</t>
-  </si>
-  <si>
-    <t>A75/6B/2 Bạch Đằng,Phường</t>
-  </si>
-  <si>
     <t>LISA</t>
   </si>
   <si>
     <t>685 tân sơn phường 12</t>
   </si>
   <si>
-    <t>004GE</t>
-  </si>
-  <si>
-    <t>159/43/5 Đường Bạch Đằng</t>
-  </si>
-  <si>
     <t>280a12 Lương Đình Của. An Phú</t>
   </si>
   <si>
@@ -1337,6 +1238,117 @@
   </si>
   <si>
     <t>gộp, đổi hàng</t>
+  </si>
+  <si>
+    <t>159/43/5 Đường Bạch Đằng, phường Tân Sơn Hòa</t>
+  </si>
+  <si>
+    <t>THU TRƯƠNG</t>
+  </si>
+  <si>
+    <t>238/3 trường chinh, đông hưng thuận</t>
+  </si>
+  <si>
+    <t>A75/6B/2 Bạch Đằng, Phường 2</t>
+  </si>
+  <si>
+    <t>FANG FANG</t>
+  </si>
+  <si>
+    <t>17-19 Trường Sơn P4</t>
+  </si>
+  <si>
+    <t>gộp</t>
+  </si>
+  <si>
+    <t>Loan Thỏ</t>
+  </si>
+  <si>
+    <t>290 an dương vương phường chợ quán</t>
+  </si>
+  <si>
+    <t>HD018248</t>
+  </si>
+  <si>
+    <t>5 lê thánh tôn bến nghé</t>
+  </si>
+  <si>
+    <t>DARAVIN</t>
+  </si>
+  <si>
+    <t>301 Phạm Ngũ Lão, Phường Phạm Ngũ Lão</t>
+  </si>
+  <si>
+    <t>30/18 đường số 6 KP18 Phường Vĩnh Hội</t>
+  </si>
+  <si>
+    <t>chung cư the park residence, 12 nguyễn hữu thọ phước kien nha be</t>
+  </si>
+  <si>
+    <t>56/41 dương ba trạc, Phường 02</t>
+  </si>
+  <si>
+    <t>yenchau</t>
+  </si>
+  <si>
+    <t>Chung cu Horita, lo C, Đường D4, P. Tân Hưng</t>
+  </si>
+  <si>
+    <t>27 nguyễn hữu thọ ( sunrise city toà X1) phường Tân Hưng</t>
+  </si>
+  <si>
+    <t>saigon mia block b cổng sau</t>
+  </si>
+  <si>
+    <t>Hiểu My</t>
+  </si>
+  <si>
+    <t>HD018563</t>
+  </si>
+  <si>
+    <t>Toà 2, chung cư river panorama, 20 lê thị chợ, phường phú thuận</t>
+  </si>
+  <si>
+    <t>Thanh Xuân</t>
+  </si>
+  <si>
+    <t>17/4B Liên khu 5-6 bình hưng hòa b</t>
+  </si>
+  <si>
+    <t>Tuyết Nhi</t>
+  </si>
+  <si>
+    <t>Nhung Bùi</t>
+  </si>
+  <si>
+    <t>409/108/32/14c huynh thị hai, tân chánh hiệp</t>
+  </si>
+  <si>
+    <t>192 Phạm Đức Sơn, Phường 16 (Chung Cư Heaven Riverview - Mỹ Phúc) Block B</t>
+  </si>
+  <si>
+    <t>HD018486</t>
+  </si>
+  <si>
+    <t>HD018435</t>
+  </si>
+  <si>
+    <t>A28/1Dw3 quốc lộ 50 ấp 1 xã bình hưng</t>
+  </si>
+  <si>
+    <t>HD018540</t>
+  </si>
+  <si>
+    <t>007 Lộ B chung cư Tây Thạnh, phường Tân Thạnh</t>
+  </si>
+  <si>
+    <t>E3/8 ấp 56 xã vĩnh lộc</t>
+  </si>
+  <si>
+    <t>536/32/23 âu cơ</t>
+  </si>
+  <si>
+    <t>17 Đường Số 13 Bình Hưng Hoà</t>
   </si>
 </sst>
 </file>
@@ -1366,7 +1378,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1402,16 +1414,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF9999"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFD0D0"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1425,7 +1427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1439,10 +1441,8 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2971,7 +2971,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I56" si="1">G35-H35</f>
         <v>30</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -4771,7 +4771,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -4779,14 +4779,14 @@
     <col min="3" max="3" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="64.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" style="13" customWidth="1"/>
     <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="4.7109375" bestFit="1" customWidth="1"/>
@@ -4816,7 +4816,7 @@
       <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -4850,613 +4850,627 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="3" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G3">
-        <v>815</v>
-      </c>
-      <c r="H3">
-        <v>25</v>
-      </c>
-      <c r="I3">
+      <c r="G3" s="6">
+        <v>790</v>
+      </c>
+      <c r="H3" s="6">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6">
         <f t="shared" ref="I3:I34" si="0">G3-H3</f>
         <v>790</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="K3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="M3" s="6" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="G4">
-        <v>480</v>
-      </c>
-      <c r="H4">
+      <c r="G4" s="8">
         <v>30</v>
       </c>
-      <c r="I4">
-        <f t="shared" si="0"/>
-        <v>450</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="H4" s="8">
+        <v>30</v>
+      </c>
+      <c r="I4" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K4" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" t="s">
+      <c r="K4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="8" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="M4" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="6">
         <v>535</v>
       </c>
-      <c r="H5">
-        <v>25</v>
-      </c>
-      <c r="I5">
+      <c r="H5" s="6">
+        <v>25</v>
+      </c>
+      <c r="I5" s="6">
         <f t="shared" si="0"/>
         <v>510</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" t="s">
+      <c r="K5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s">
+    <row r="6" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="8">
         <v>915</v>
       </c>
-      <c r="H6">
-        <v>25</v>
-      </c>
-      <c r="I6">
+      <c r="H6" s="8">
+        <v>25</v>
+      </c>
+      <c r="I6" s="8">
         <f t="shared" si="0"/>
         <v>890</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" t="s">
+      <c r="K6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="8" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
+    <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G7" s="6">
+        <v>820</v>
+      </c>
+      <c r="H7" s="6">
+        <v>30</v>
+      </c>
+      <c r="I7" s="6">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="8">
+        <v>850</v>
+      </c>
+      <c r="H8" s="8">
+        <v>30</v>
+      </c>
+      <c r="I8" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="D9" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="G7">
-        <v>790</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <f t="shared" si="0"/>
-        <v>790</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="E9" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="G9" s="6">
+        <v>2620</v>
+      </c>
+      <c r="H9" s="6">
+        <v>30</v>
+      </c>
+      <c r="I9" s="6">
+        <f t="shared" si="0"/>
+        <v>2590</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="8">
+        <v>670</v>
+      </c>
+      <c r="H10" s="8">
+        <v>30</v>
+      </c>
+      <c r="I10" s="8">
+        <f t="shared" si="0"/>
+        <v>640</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L7" t="s">
+      <c r="K10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="8" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>302</v>
-      </c>
-      <c r="D8" t="s">
-        <v>303</v>
-      </c>
-      <c r="E8" t="s">
-        <v>304</v>
-      </c>
-      <c r="F8" s="14" t="s">
+    <row r="11" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="G8">
+      <c r="D11" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="6">
+        <v>705</v>
+      </c>
+      <c r="H11" s="6">
+        <v>35</v>
+      </c>
+      <c r="I11" s="6">
+        <f t="shared" si="0"/>
+        <v>670</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G12" s="6">
+        <v>2860</v>
+      </c>
+      <c r="H12" s="6">
+        <v>30</v>
+      </c>
+      <c r="I12" s="6">
+        <f t="shared" si="0"/>
+        <v>2830</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="8">
+        <v>1515</v>
+      </c>
+      <c r="H13" s="8">
+        <v>35</v>
+      </c>
+      <c r="I13" s="8">
+        <f t="shared" si="0"/>
+        <v>1480</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="8">
+        <v>690</v>
+      </c>
+      <c r="H14" s="8">
+        <v>30</v>
+      </c>
+      <c r="I14" s="8">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="G15" s="6">
+        <v>1165</v>
+      </c>
+      <c r="H15" s="6">
+        <v>25</v>
+      </c>
+      <c r="I15" s="6">
+        <f t="shared" si="0"/>
+        <v>1140</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G16" s="6">
+        <v>1350</v>
+      </c>
+      <c r="H16" s="6">
+        <v>30</v>
+      </c>
+      <c r="I16" s="6">
+        <f t="shared" si="0"/>
+        <v>1320</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="8">
+        <v>1345</v>
+      </c>
+      <c r="H17" s="8">
+        <v>25</v>
+      </c>
+      <c r="I17" s="8">
+        <f t="shared" si="0"/>
+        <v>1320</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="6">
+        <v>675</v>
+      </c>
+      <c r="H18" s="6">
+        <v>35</v>
+      </c>
+      <c r="I18" s="6">
+        <f t="shared" si="0"/>
+        <v>640</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" s="8">
+        <v>850</v>
+      </c>
+      <c r="H19" s="8">
+        <v>30</v>
+      </c>
+      <c r="I19" s="8">
+        <f t="shared" si="0"/>
         <v>820</v>
       </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <f t="shared" si="0"/>
-        <v>820</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="J19" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L8" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" t="s">
-        <v>306</v>
-      </c>
-      <c r="D9" t="s">
-        <v>307</v>
-      </c>
-      <c r="E9" t="s">
-        <v>308</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>309</v>
-      </c>
-      <c r="G9">
-        <v>2645</v>
-      </c>
-      <c r="H9">
-        <v>25</v>
-      </c>
-      <c r="I9">
-        <f t="shared" si="0"/>
-        <v>2620</v>
-      </c>
-      <c r="J9" t="s">
-        <v>37</v>
-      </c>
-      <c r="K9" t="s">
-        <v>24</v>
-      </c>
-      <c r="L9" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>310</v>
-      </c>
-      <c r="D10" t="s">
-        <v>311</v>
-      </c>
-      <c r="E10" t="s">
-        <v>312</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10">
-        <v>670</v>
-      </c>
-      <c r="H10">
-        <v>30</v>
-      </c>
-      <c r="I10">
-        <f t="shared" si="0"/>
-        <v>640</v>
-      </c>
-      <c r="J10" t="s">
-        <v>291</v>
-      </c>
-      <c r="K10" t="s">
-        <v>24</v>
-      </c>
-      <c r="L10" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>313</v>
-      </c>
-      <c r="D11" t="s">
-        <v>314</v>
-      </c>
-      <c r="E11" t="s">
-        <v>315</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="G11">
-        <v>705</v>
-      </c>
-      <c r="H11">
-        <v>35</v>
-      </c>
-      <c r="I11">
-        <f t="shared" si="0"/>
-        <v>670</v>
-      </c>
-      <c r="J11" t="s">
-        <v>291</v>
-      </c>
-      <c r="K11" t="s">
-        <v>24</v>
-      </c>
-      <c r="L11" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" t="s">
-        <v>316</v>
-      </c>
-      <c r="D12" t="s">
-        <v>317</v>
-      </c>
-      <c r="E12" t="s">
-        <v>318</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G12">
-        <v>2885</v>
-      </c>
-      <c r="H12">
-        <v>25</v>
-      </c>
-      <c r="I12">
-        <f t="shared" si="0"/>
-        <v>2860</v>
-      </c>
-      <c r="J12" t="s">
-        <v>37</v>
-      </c>
-      <c r="K12" t="s">
-        <v>24</v>
-      </c>
-      <c r="L12" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" t="s">
-        <v>319</v>
-      </c>
-      <c r="D13" s="13"/>
-      <c r="E13" t="s">
-        <v>320</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13">
-        <v>1481</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
-        <f t="shared" si="0"/>
-        <v>1480</v>
-      </c>
-      <c r="J13" t="s">
-        <v>37</v>
-      </c>
-      <c r="K13" t="s">
-        <v>24</v>
-      </c>
-      <c r="L13" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" t="s">
-        <v>321</v>
-      </c>
-      <c r="D14" t="s">
-        <v>322</v>
-      </c>
-      <c r="E14" t="s">
-        <v>323</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="G14">
-        <v>690</v>
-      </c>
-      <c r="H14">
-        <v>30</v>
-      </c>
-      <c r="I14">
-        <f t="shared" si="0"/>
-        <v>660</v>
-      </c>
-      <c r="J14" t="s">
-        <v>291</v>
-      </c>
-      <c r="K14" t="s">
-        <v>24</v>
-      </c>
-      <c r="L14" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" t="s">
-        <v>324</v>
-      </c>
-      <c r="D15" t="s">
-        <v>325</v>
-      </c>
-      <c r="E15" t="s">
-        <v>326</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="G15">
-        <v>1165</v>
-      </c>
-      <c r="H15">
-        <v>25</v>
-      </c>
-      <c r="I15">
-        <f t="shared" si="0"/>
-        <v>1140</v>
-      </c>
-      <c r="J15" t="s">
-        <v>37</v>
-      </c>
-      <c r="K15" t="s">
-        <v>24</v>
-      </c>
-      <c r="L15" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" t="s">
-        <v>327</v>
-      </c>
-      <c r="D16" t="s">
-        <v>328</v>
-      </c>
-      <c r="E16" t="s">
-        <v>329</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="G16">
-        <v>1350</v>
-      </c>
-      <c r="H16">
-        <v>30</v>
-      </c>
-      <c r="I16">
-        <f t="shared" si="0"/>
-        <v>1320</v>
-      </c>
-      <c r="J16" t="s">
-        <v>291</v>
-      </c>
-      <c r="K16" t="s">
-        <v>24</v>
-      </c>
-      <c r="L16" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" t="s">
-        <v>330</v>
-      </c>
-      <c r="D17" t="s">
-        <v>331</v>
-      </c>
-      <c r="E17" t="s">
-        <v>332</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G17">
-        <v>1345</v>
-      </c>
-      <c r="H17">
-        <v>25</v>
-      </c>
-      <c r="I17">
-        <f t="shared" si="0"/>
-        <v>1320</v>
-      </c>
-      <c r="J17" t="s">
-        <v>37</v>
-      </c>
-      <c r="K17" t="s">
-        <v>24</v>
-      </c>
-      <c r="L17" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" t="s">
-        <v>333</v>
-      </c>
-      <c r="D18" t="s">
-        <v>334</v>
-      </c>
-      <c r="E18" t="s">
-        <v>335</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G18">
-        <v>670</v>
-      </c>
-      <c r="H18">
-        <v>30</v>
-      </c>
-      <c r="I18">
-        <f t="shared" si="0"/>
-        <v>640</v>
-      </c>
-      <c r="J18" t="s">
-        <v>291</v>
-      </c>
-      <c r="K18" t="s">
-        <v>24</v>
-      </c>
-      <c r="L18" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" t="s">
-        <v>336</v>
-      </c>
-      <c r="D19" t="s">
-        <v>337</v>
-      </c>
-      <c r="E19" t="s">
-        <v>338</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19">
-        <v>850</v>
-      </c>
-      <c r="H19">
-        <v>30</v>
-      </c>
-      <c r="I19">
-        <f t="shared" si="0"/>
-        <v>820</v>
-      </c>
-      <c r="J19" t="s">
-        <v>291</v>
-      </c>
-      <c r="K19" t="s">
-        <v>24</v>
-      </c>
-      <c r="L19" t="s">
+      <c r="K19" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="8" t="s">
         <v>287</v>
       </c>
     </row>
@@ -5465,26 +5479,26 @@
         <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>430</v>
+        <v>397</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>431</v>
+        <v>398</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>48</v>
       </c>
       <c r="G20" s="3">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H20" s="3">
         <v>0</v>
       </c>
       <c r="I20" s="3">
         <f t="shared" si="0"/>
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>24</v>
@@ -5496,42 +5510,42 @@
         <v>287</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" t="s">
-        <v>340</v>
-      </c>
-      <c r="D21" t="s">
-        <v>341</v>
-      </c>
-      <c r="E21" t="s">
-        <v>342</v>
-      </c>
-      <c r="F21" s="14" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F21" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="8">
         <v>830</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="8">
         <v>30</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="8">
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K21" t="s">
-        <v>24</v>
-      </c>
-      <c r="L21" t="s">
+      <c r="K21" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="8" t="s">
         <v>287</v>
       </c>
     </row>
@@ -5540,13 +5554,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>426</v>
+        <v>393</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>48</v>
@@ -5571,361 +5585,366 @@
         <v>287</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" t="s">
+    <row r="23" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G23" s="3">
+        <v>820</v>
+      </c>
+      <c r="H23" s="3">
+        <v>20</v>
+      </c>
+      <c r="I23" s="3">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="G24" s="6">
+        <v>660</v>
+      </c>
+      <c r="H24" s="6">
+        <v>20</v>
+      </c>
+      <c r="I24" s="6">
+        <f t="shared" si="0"/>
+        <v>640</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G25" s="6">
+        <v>1430</v>
+      </c>
+      <c r="H25" s="6">
+        <v>30</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="0"/>
+        <v>1400</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G26" s="6">
+        <v>775</v>
+      </c>
+      <c r="H26" s="6">
+        <v>25</v>
+      </c>
+      <c r="I26" s="6">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="8">
+        <v>0</v>
+      </c>
+      <c r="H27" s="8">
+        <v>25</v>
+      </c>
+      <c r="I27" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E28" s="8" t="s">
         <v>346</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F28" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" s="8">
+        <v>780</v>
+      </c>
+      <c r="H28" s="8">
+        <v>30</v>
+      </c>
+      <c r="I28" s="8">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="F23" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="G23">
+      <c r="E29" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G29" s="6">
+        <v>855</v>
+      </c>
+      <c r="H29" s="6">
+        <v>35</v>
+      </c>
+      <c r="I29" s="6">
+        <f t="shared" si="0"/>
         <v>820</v>
       </c>
-      <c r="H23">
-        <v>20</v>
-      </c>
-      <c r="I23">
-        <f t="shared" si="0"/>
-        <v>800</v>
-      </c>
-      <c r="J23" t="s">
-        <v>24</v>
-      </c>
-      <c r="K23" t="s">
-        <v>24</v>
-      </c>
-      <c r="L23" t="s">
+      <c r="J29" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" t="s">
+    <row r="30" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D30" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E30" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F30" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G30" s="8">
+        <v>740</v>
+      </c>
+      <c r="H30" s="8">
+        <v>30</v>
+      </c>
+      <c r="I30" s="8">
+        <f t="shared" si="0"/>
+        <v>710</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="G24">
-        <v>660</v>
-      </c>
-      <c r="H24">
-        <v>20</v>
-      </c>
-      <c r="I24">
-        <f t="shared" si="0"/>
-        <v>640</v>
-      </c>
-      <c r="J24" t="s">
-        <v>37</v>
-      </c>
-      <c r="K24" t="s">
-        <v>24</v>
-      </c>
-      <c r="L24" t="s">
+      <c r="D31" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" s="3">
+        <v>2120</v>
+      </c>
+      <c r="H31" s="3">
+        <v>35</v>
+      </c>
+      <c r="I31" s="3">
+        <f t="shared" si="0"/>
+        <v>2085</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="3" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" t="s">
-        <v>352</v>
-      </c>
-      <c r="D25" t="s">
-        <v>353</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="M31" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="G25">
-        <v>1430</v>
-      </c>
-      <c r="H25">
-        <v>30</v>
-      </c>
-      <c r="I25">
-        <f t="shared" si="0"/>
-        <v>1400</v>
-      </c>
-      <c r="J25" t="s">
+      <c r="D32" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G32" s="8">
+        <v>755</v>
+      </c>
+      <c r="H32" s="8">
+        <v>25</v>
+      </c>
+      <c r="I32" s="8">
+        <f t="shared" si="0"/>
+        <v>730</v>
+      </c>
+      <c r="J32" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K25" t="s">
-        <v>24</v>
-      </c>
-      <c r="L25" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" t="s">
-        <v>284</v>
-      </c>
-      <c r="D26" t="s">
-        <v>355</v>
-      </c>
-      <c r="E26" t="s">
-        <v>286</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="G26">
-        <v>775</v>
-      </c>
-      <c r="H26">
-        <v>25</v>
-      </c>
-      <c r="I26">
-        <f t="shared" si="0"/>
-        <v>750</v>
-      </c>
-      <c r="J26" t="s">
-        <v>37</v>
-      </c>
-      <c r="K26" t="s">
-        <v>24</v>
-      </c>
-      <c r="L26" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" t="s">
-        <v>356</v>
-      </c>
-      <c r="D27" s="13"/>
-      <c r="E27" t="s">
-        <v>357</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="G27">
-        <v>124</v>
-      </c>
-      <c r="H27">
-        <v>25</v>
-      </c>
-      <c r="I27">
-        <f t="shared" si="0"/>
-        <v>99</v>
-      </c>
-      <c r="J27" t="s">
-        <v>291</v>
-      </c>
-      <c r="K27" t="s">
-        <v>24</v>
-      </c>
-      <c r="L27" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>18</v>
-      </c>
-      <c r="C28" t="s">
-        <v>358</v>
-      </c>
-      <c r="D28" t="s">
-        <v>359</v>
-      </c>
-      <c r="E28" t="s">
-        <v>360</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28">
-        <v>780</v>
-      </c>
-      <c r="H28">
-        <v>30</v>
-      </c>
-      <c r="I28">
-        <f t="shared" si="0"/>
-        <v>750</v>
-      </c>
-      <c r="J28" t="s">
-        <v>291</v>
-      </c>
-      <c r="K28" t="s">
-        <v>24</v>
-      </c>
-      <c r="L28" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>18</v>
-      </c>
-      <c r="C29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D29" t="s">
-        <v>361</v>
-      </c>
-      <c r="E29" t="s">
-        <v>362</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G29">
-        <v>855</v>
-      </c>
-      <c r="H29">
-        <v>35</v>
-      </c>
-      <c r="I29">
-        <f t="shared" si="0"/>
-        <v>820</v>
-      </c>
-      <c r="J29" t="s">
-        <v>291</v>
-      </c>
-      <c r="K29" t="s">
-        <v>24</v>
-      </c>
-      <c r="L29" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" t="s">
-        <v>363</v>
-      </c>
-      <c r="D30" t="s">
-        <v>364</v>
-      </c>
-      <c r="E30" t="s">
-        <v>365</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="G30">
-        <v>2090</v>
-      </c>
-      <c r="H30">
-        <v>710</v>
-      </c>
-      <c r="I30">
-        <f t="shared" si="0"/>
-        <v>1380</v>
-      </c>
-      <c r="J30" t="s">
-        <v>291</v>
-      </c>
-      <c r="K30" t="s">
-        <v>24</v>
-      </c>
-      <c r="L30" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" t="s">
-        <v>366</v>
-      </c>
-      <c r="D31" t="s">
-        <v>367</v>
-      </c>
-      <c r="E31" t="s">
-        <v>368</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G31">
-        <v>2150</v>
-      </c>
-      <c r="H31">
-        <v>30</v>
-      </c>
-      <c r="I31">
-        <f t="shared" si="0"/>
-        <v>2120</v>
-      </c>
-      <c r="J31" t="s">
-        <v>24</v>
-      </c>
-      <c r="K31" t="s">
-        <v>24</v>
-      </c>
-      <c r="L31" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>18</v>
-      </c>
-      <c r="C32" t="s">
-        <v>369</v>
-      </c>
-      <c r="D32" t="s">
-        <v>370</v>
-      </c>
-      <c r="E32" t="s">
-        <v>371</v>
-      </c>
-      <c r="F32" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G32">
-        <v>755</v>
-      </c>
-      <c r="H32">
-        <v>25</v>
-      </c>
-      <c r="I32">
-        <f t="shared" si="0"/>
-        <v>730</v>
-      </c>
-      <c r="J32" t="s">
-        <v>37</v>
-      </c>
-      <c r="K32" t="s">
-        <v>24</v>
-      </c>
-      <c r="L32" t="s">
+      <c r="K32" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="8" t="s">
         <v>287</v>
       </c>
     </row>
@@ -5934,15 +5953,15 @@
         <v>18</v>
       </c>
       <c r="C33" t="s">
-        <v>372</v>
+        <v>356</v>
       </c>
       <c r="D33" t="s">
-        <v>373</v>
+        <v>357</v>
       </c>
       <c r="E33" t="s">
-        <v>374</v>
-      </c>
-      <c r="F33" s="14" t="s">
+        <v>358</v>
+      </c>
+      <c r="F33" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G33">
@@ -5970,13 +5989,13 @@
         <v>18</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>430</v>
+        <v>397</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>375</v>
+        <v>359</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>431</v>
+        <v>398</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>48</v>
@@ -6001,254 +6020,261 @@
         <v>287</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" t="s">
-        <v>376</v>
-      </c>
-      <c r="D35" t="s">
-        <v>377</v>
-      </c>
-      <c r="E35" t="s">
-        <v>378</v>
-      </c>
-      <c r="F35" s="14" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G35">
-        <v>2145</v>
-      </c>
-      <c r="H35">
-        <v>25</v>
-      </c>
-      <c r="I35">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+      <c r="G35" s="6">
         <v>2120</v>
       </c>
-      <c r="J35" t="s">
+      <c r="H35" s="6">
+        <v>30</v>
+      </c>
+      <c r="I35" s="6">
+        <f t="shared" ref="I35:I54" si="1">G35-H35</f>
+        <v>2090</v>
+      </c>
+      <c r="J35" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K35" t="s">
-        <v>24</v>
-      </c>
-      <c r="L35" t="s">
+      <c r="K35" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L35" s="6" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>18</v>
-      </c>
-      <c r="C36" t="s">
-        <v>379</v>
-      </c>
-      <c r="D36" t="s">
-        <v>380</v>
-      </c>
-      <c r="E36" t="s">
-        <v>381</v>
-      </c>
-      <c r="F36" s="14" t="s">
+      <c r="M35" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="G36">
-        <v>850</v>
-      </c>
-      <c r="H36">
+      <c r="G36" s="6">
+        <v>0</v>
+      </c>
+      <c r="H36" s="6">
         <v>30</v>
       </c>
-      <c r="I36">
+      <c r="I36" s="6">
         <f t="shared" si="1"/>
-        <v>820</v>
-      </c>
-      <c r="J36" t="s">
-        <v>291</v>
-      </c>
-      <c r="K36" t="s">
-        <v>24</v>
-      </c>
-      <c r="L36" t="s">
+        <v>-30</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>18</v>
-      </c>
-      <c r="C37" t="s">
-        <v>382</v>
-      </c>
-      <c r="D37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E37" t="s">
-        <v>384</v>
-      </c>
-      <c r="F37" s="16"/>
-      <c r="G37">
-        <v>510</v>
-      </c>
-      <c r="H37">
-        <v>0</v>
-      </c>
-      <c r="I37">
+    <row r="37" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G37" s="6">
+        <v>535</v>
+      </c>
+      <c r="H37" s="6">
+        <v>25</v>
+      </c>
+      <c r="I37" s="6">
         <f t="shared" si="1"/>
         <v>510</v>
       </c>
-      <c r="J37" t="s">
-        <v>291</v>
-      </c>
-      <c r="K37" t="s">
-        <v>24</v>
-      </c>
-      <c r="L37" t="s">
+      <c r="J37" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L37" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
-        <v>18</v>
-      </c>
-      <c r="C38" t="s">
-        <v>385</v>
-      </c>
-      <c r="D38" t="s">
-        <v>386</v>
-      </c>
-      <c r="E38" t="s">
-        <v>387</v>
-      </c>
-      <c r="F38" s="16"/>
-      <c r="G38">
-        <v>700</v>
-      </c>
-      <c r="H38">
-        <v>0</v>
-      </c>
-      <c r="I38">
+    <row r="38" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="8">
+        <v>735</v>
+      </c>
+      <c r="H38" s="8">
+        <v>35</v>
+      </c>
+      <c r="I38" s="8">
         <f t="shared" si="1"/>
         <v>700</v>
       </c>
-      <c r="J38" t="s">
+      <c r="J38" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K38" t="s">
-        <v>24</v>
-      </c>
-      <c r="L38" t="s">
+      <c r="K38" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L38" s="8" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" t="s">
-        <v>388</v>
-      </c>
-      <c r="D39" t="s">
-        <v>389</v>
-      </c>
-      <c r="E39" t="s">
-        <v>390</v>
-      </c>
-      <c r="F39" s="14" t="s">
+    <row r="39" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="G39">
-        <v>375</v>
-      </c>
-      <c r="H39">
-        <v>25</v>
-      </c>
-      <c r="I39">
+      <c r="G39" s="6">
+        <v>0</v>
+      </c>
+      <c r="H39" s="6">
+        <v>25</v>
+      </c>
+      <c r="I39" s="6">
         <f t="shared" si="1"/>
-        <v>350</v>
-      </c>
-      <c r="J39" t="s">
+        <v>-25</v>
+      </c>
+      <c r="J39" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K39" t="s">
-        <v>24</v>
-      </c>
-      <c r="L39" t="s">
+      <c r="K39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L39" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B40" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40" t="s">
-        <v>391</v>
-      </c>
-      <c r="D40" t="s">
-        <v>392</v>
-      </c>
-      <c r="E40" t="s">
-        <v>393</v>
-      </c>
-      <c r="F40" s="14" t="s">
+    <row r="40" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F40" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="6">
         <v>1355</v>
       </c>
-      <c r="H40">
-        <v>25</v>
-      </c>
-      <c r="I40">
+      <c r="H40" s="6">
+        <v>25</v>
+      </c>
+      <c r="I40" s="6">
         <f t="shared" si="1"/>
         <v>1330</v>
       </c>
-      <c r="J40" t="s">
+      <c r="J40" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K40" t="s">
-        <v>24</v>
-      </c>
-      <c r="L40" t="s">
+      <c r="K40" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L40" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
-        <v>18</v>
-      </c>
-      <c r="C41" t="s">
-        <v>394</v>
-      </c>
-      <c r="D41" t="s">
-        <v>395</v>
-      </c>
-      <c r="E41" t="s">
-        <v>396</v>
-      </c>
-      <c r="F41" s="14" t="s">
+    <row r="41" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="F41" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="6">
         <v>1890</v>
       </c>
-      <c r="H41">
+      <c r="H41" s="6">
         <v>30</v>
       </c>
-      <c r="I41">
+      <c r="I41" s="6">
         <f t="shared" si="1"/>
         <v>1860</v>
       </c>
-      <c r="J41" t="s">
-        <v>291</v>
-      </c>
-      <c r="K41" t="s">
-        <v>24</v>
-      </c>
-      <c r="L41" t="s">
+      <c r="J41" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L41" s="6" t="s">
         <v>287</v>
       </c>
     </row>
@@ -6257,13 +6283,13 @@
         <v>18</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>397</v>
+        <v>374</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>398</v>
+        <v>375</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>399</v>
+        <v>376</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>29</v>
@@ -6293,13 +6319,13 @@
         <v>18</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>400</v>
+        <v>377</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>401</v>
+        <v>378</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>402</v>
+        <v>379</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>81</v>
@@ -6327,179 +6353,186 @@
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>18</v>
-      </c>
-      <c r="C44" t="s">
-        <v>403</v>
-      </c>
-      <c r="D44" t="s">
-        <v>404</v>
-      </c>
-      <c r="E44" t="s">
-        <v>405</v>
-      </c>
-      <c r="F44" s="16"/>
-      <c r="G44">
-        <v>790</v>
-      </c>
-      <c r="H44">
+    <row r="44" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G44" s="8">
         <v>0</v>
       </c>
-      <c r="I44">
+      <c r="H44" s="8">
+        <v>30</v>
+      </c>
+      <c r="I44" s="8">
         <f t="shared" si="1"/>
-        <v>790</v>
-      </c>
-      <c r="J44" t="s">
+        <v>-30</v>
+      </c>
+      <c r="J44" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K44" t="s">
-        <v>24</v>
-      </c>
-      <c r="L44" t="s">
+      <c r="K44" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L44" s="8" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B45" t="s">
-        <v>18</v>
-      </c>
-      <c r="C45" t="s">
-        <v>406</v>
-      </c>
-      <c r="D45" t="s">
+    <row r="45" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G45" s="3">
+        <v>0</v>
+      </c>
+      <c r="H45" s="3">
+        <v>30</v>
+      </c>
+      <c r="I45" s="3">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K45" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L45" s="3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G46" s="6">
+        <v>30</v>
+      </c>
+      <c r="H46" s="6">
+        <v>30</v>
+      </c>
+      <c r="I46" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L46" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="M46" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="E45" t="s">
-        <v>408</v>
-      </c>
-      <c r="F45" s="16"/>
-      <c r="G45">
-        <v>1520</v>
-      </c>
-      <c r="H45">
+      <c r="D47" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="G47" s="6">
+        <v>25</v>
+      </c>
+      <c r="H47" s="6">
+        <v>25</v>
+      </c>
+      <c r="I47" s="6">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I45">
-        <f t="shared" si="1"/>
-        <v>1520</v>
-      </c>
-      <c r="J45" t="s">
-        <v>291</v>
-      </c>
-      <c r="K45" t="s">
-        <v>24</v>
-      </c>
-      <c r="L45" t="s">
+      <c r="J47" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L47" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B46" t="s">
-        <v>18</v>
-      </c>
-      <c r="C46" t="s">
-        <v>162</v>
-      </c>
-      <c r="D46" t="s">
-        <v>409</v>
-      </c>
-      <c r="E46" t="s">
-        <v>164</v>
-      </c>
-      <c r="F46" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="G46">
-        <v>770</v>
-      </c>
-      <c r="H46">
+    <row r="48" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G48" s="8">
+        <v>690</v>
+      </c>
+      <c r="H48" s="8">
         <v>30</v>
       </c>
-      <c r="I46">
-        <f t="shared" si="1"/>
-        <v>740</v>
-      </c>
-      <c r="J46" t="s">
-        <v>291</v>
-      </c>
-      <c r="K46" t="s">
-        <v>24</v>
-      </c>
-      <c r="L46" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B47" t="s">
-        <v>18</v>
-      </c>
-      <c r="C47" t="s">
-        <v>410</v>
-      </c>
-      <c r="D47" t="s">
-        <v>411</v>
-      </c>
-      <c r="E47" t="s">
-        <v>412</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>309</v>
-      </c>
-      <c r="G47">
-        <v>475</v>
-      </c>
-      <c r="H47">
-        <v>25</v>
-      </c>
-      <c r="I47">
-        <f t="shared" si="1"/>
-        <v>450</v>
-      </c>
-      <c r="J47" t="s">
-        <v>37</v>
-      </c>
-      <c r="K47" t="s">
-        <v>24</v>
-      </c>
-      <c r="L47" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>18</v>
-      </c>
-      <c r="C48" t="s">
-        <v>413</v>
-      </c>
-      <c r="D48" t="s">
-        <v>414</v>
-      </c>
-      <c r="E48" t="s">
-        <v>415</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="G48">
-        <v>690</v>
-      </c>
-      <c r="H48">
-        <v>30</v>
-      </c>
-      <c r="I48">
+      <c r="I48" s="8">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K48" t="s">
-        <v>24</v>
-      </c>
-      <c r="L48" t="s">
+      <c r="K48" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L48" s="8" t="s">
         <v>287</v>
       </c>
     </row>
@@ -6508,13 +6541,13 @@
         <v>18</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>416</v>
+        <v>388</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>417</v>
+        <v>389</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>427</v>
+        <v>394</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>70</v>
@@ -6539,77 +6572,75 @@
         <v>287</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="B50" t="s">
-        <v>18</v>
-      </c>
-      <c r="C50" t="s">
-        <v>418</v>
-      </c>
-      <c r="D50" s="13"/>
-      <c r="E50" t="s">
-        <v>419</v>
-      </c>
-      <c r="F50" s="14" t="s">
+      <c r="B50" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="F50" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="8">
         <v>0</v>
       </c>
-      <c r="H50">
+      <c r="H50" s="8">
+        <v>35</v>
+      </c>
+      <c r="I50" s="8">
+        <f t="shared" si="1"/>
+        <v>-35</v>
+      </c>
+      <c r="J50" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K50" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L50" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G51" s="6">
+        <v>750</v>
+      </c>
+      <c r="H51" s="6">
         <v>30</v>
       </c>
-      <c r="I50">
+      <c r="I51" s="6">
         <f t="shared" si="1"/>
-        <v>-30</v>
-      </c>
-      <c r="J50" t="s">
-        <v>291</v>
-      </c>
-      <c r="K50" t="s">
-        <v>24</v>
-      </c>
-      <c r="L50" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>193</v>
-      </c>
-      <c r="B51" t="s">
-        <v>18</v>
-      </c>
-      <c r="C51" t="s">
-        <v>420</v>
-      </c>
-      <c r="D51" s="13"/>
-      <c r="E51" t="s">
-        <v>421</v>
-      </c>
-      <c r="F51" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G51">
-        <v>0</v>
-      </c>
-      <c r="H51">
         <v>720</v>
       </c>
-      <c r="I51">
-        <f t="shared" si="1"/>
-        <v>-720</v>
-      </c>
-      <c r="J51" t="s">
+      <c r="J51" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K51" t="s">
-        <v>24</v>
-      </c>
-      <c r="L51" t="s">
+      <c r="K51" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L51" s="6" t="s">
         <v>287</v>
       </c>
     </row>
@@ -6621,10 +6652,10 @@
         <v>18</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>428</v>
+        <v>395</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>429</v>
+        <v>396</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>70</v>
@@ -6657,10 +6688,10 @@
         <v>18</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>422</v>
+        <v>391</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>423</v>
+        <v>392</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>70</v>
@@ -6685,44 +6716,116 @@
         <v>287</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="B54" t="s">
-        <v>18</v>
-      </c>
-      <c r="C54" t="s">
-        <v>424</v>
-      </c>
-      <c r="D54" s="13"/>
-      <c r="E54" t="s">
-        <v>425</v>
-      </c>
-      <c r="F54" s="14" t="s">
+      <c r="B54" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="F54" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="G54">
+      <c r="G54" s="3">
+        <v>40</v>
+      </c>
+      <c r="H54" s="3">
+        <v>40</v>
+      </c>
+      <c r="I54" s="3">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H54">
-        <v>25</v>
-      </c>
-      <c r="I54">
-        <f t="shared" si="1"/>
-        <v>-25</v>
-      </c>
-      <c r="J54" t="s">
+      <c r="J54" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K54" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L54" s="3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G55" s="6">
+        <v>30</v>
+      </c>
+      <c r="H55" s="6">
+        <v>30</v>
+      </c>
+      <c r="I55" s="6">
+        <f t="shared" ref="I55:I56" si="2">G55-H55</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K54" t="s">
-        <v>24</v>
-      </c>
-      <c r="L54" t="s">
+      <c r="K55" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L55" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G56" s="8">
+        <v>770</v>
+      </c>
+      <c r="H56" s="8">
+        <v>30</v>
+      </c>
+      <c r="I56" s="8">
+        <f t="shared" si="2"/>
+        <v>740</v>
+      </c>
+      <c r="J56" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="K56" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L56" s="8" t="s">
         <v>287</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update report and logic for tienHang
</commit_message>
<xml_diff>
--- a/data/May/Data.xlsx
+++ b/data/May/Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\May\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D1725FD-408C-4A72-9502-2DE738FD0946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F97D96-D690-45D3-8B33-49D64547999A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="434">
   <si>
     <t>THU 6</t>
   </si>
@@ -1106,15 +1106,6 @@
   </si>
   <si>
     <t>HD018437</t>
-  </si>
-  <si>
-    <t>CN</t>
-  </si>
-  <si>
-    <t>HD000268</t>
-  </si>
-  <si>
-    <t>141/12 Âu Dương Lân</t>
   </si>
   <si>
     <t>HD018546</t>
@@ -4771,7 +4762,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P56"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -4886,7 +4877,7 @@
         <v>287</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -5011,7 +5002,7 @@
         <v>299</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>131</v>
@@ -5041,13 +5032,13 @@
         <v>18</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>131</v>
@@ -5116,13 +5107,13 @@
         <v>18</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>304</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>29</v>
@@ -5158,7 +5149,7 @@
         <v>306</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>52</v>
@@ -5194,7 +5185,7 @@
         <v>308</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>102</v>
@@ -5230,10 +5221,10 @@
         <v>309</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>52</v>
@@ -5479,13 +5470,13 @@
         <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>328</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>48</v>
@@ -5510,7 +5501,7 @@
         <v>287</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="21" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -5518,7 +5509,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>329</v>
@@ -5560,7 +5551,7 @@
         <v>332</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>48</v>
@@ -5668,7 +5659,7 @@
         <v>341</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>41</v>
@@ -5737,10 +5728,10 @@
         <v>343</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>85</v>
@@ -5812,7 +5803,7 @@
         <v>347</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>36</v>
@@ -5923,7 +5914,7 @@
         <v>355</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>102</v>
@@ -5948,39 +5939,39 @@
         <v>287</v>
       </c>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" t="s">
-        <v>356</v>
-      </c>
-      <c r="D33" t="s">
-        <v>357</v>
-      </c>
-      <c r="E33" t="s">
-        <v>358</v>
-      </c>
-      <c r="F33" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G33">
-        <v>7310</v>
-      </c>
-      <c r="H33">
+    <row r="33" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G33" s="8">
+        <v>770</v>
+      </c>
+      <c r="H33" s="8">
         <v>30</v>
       </c>
-      <c r="I33">
-        <f t="shared" si="0"/>
-        <v>7280</v>
-      </c>
-      <c r="J33" t="s">
+      <c r="I33" s="8">
+        <f>G33-H33</f>
+        <v>740</v>
+      </c>
+      <c r="J33" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="K33" t="s">
-        <v>24</v>
-      </c>
-      <c r="L33" t="s">
+      <c r="K33" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="8" t="s">
         <v>287</v>
       </c>
     </row>
@@ -5989,13 +5980,13 @@
         <v>18</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>48</v>
@@ -6020,7 +6011,7 @@
         <v>287</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="35" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -6028,13 +6019,13 @@
         <v>18</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>59</v>
@@ -6067,13 +6058,13 @@
         <v>18</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>131</v>
@@ -6103,13 +6094,13 @@
         <v>18</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>63</v>
@@ -6139,13 +6130,13 @@
         <v>18</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>52</v>
@@ -6175,13 +6166,13 @@
         <v>18</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>63</v>
@@ -6211,13 +6202,13 @@
         <v>18</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>186</v>
@@ -6247,13 +6238,13 @@
         <v>18</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>131</v>
@@ -6283,13 +6274,13 @@
         <v>18</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>29</v>
@@ -6319,13 +6310,13 @@
         <v>18</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>81</v>
@@ -6358,13 +6349,13 @@
         <v>18</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>22</v>
@@ -6394,13 +6385,13 @@
         <v>18</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>29</v>
@@ -6433,7 +6424,7 @@
         <v>162</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>164</v>
@@ -6469,13 +6460,13 @@
         <v>18</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>303</v>
@@ -6505,13 +6496,13 @@
         <v>18</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>41</v>
@@ -6541,13 +6532,13 @@
         <v>18</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>70</v>
@@ -6580,10 +6571,10 @@
         <v>18</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>22</v>
@@ -6616,10 +6607,10 @@
         <v>18</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>102</v>
@@ -6652,10 +6643,10 @@
         <v>18</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>70</v>
@@ -6688,10 +6679,10 @@
         <v>18</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>70</v>
@@ -6724,10 +6715,10 @@
         <v>18</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>102</v>
@@ -6760,10 +6751,10 @@
         <v>18</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>63</v>
@@ -6775,7 +6766,7 @@
         <v>30</v>
       </c>
       <c r="I55" s="6">
-        <f t="shared" ref="I55:I56" si="2">G55-H55</f>
+        <f t="shared" ref="I55" si="2">G55-H55</f>
         <v>0</v>
       </c>
       <c r="J55" s="6" t="s">
@@ -6785,42 +6776,6 @@
         <v>24</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C56" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>429</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G56" s="8">
-        <v>770</v>
-      </c>
-      <c r="H56" s="8">
-        <v>30</v>
-      </c>
-      <c r="I56" s="8">
-        <f t="shared" si="2"/>
-        <v>740</v>
-      </c>
-      <c r="J56" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="K56" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L56" s="8" t="s">
         <v>287</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update logic and 07-05 report
</commit_message>
<xml_diff>
--- a/data/May/Data.xlsx
+++ b/data/May/Data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778ACD3D-4F74-4ADE-87CA-5F728584095E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D04FA7-719E-4BF6-A9B0-EE591558279F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-05" sheetId="4" r:id="rId1"/>
     <sheet name="04-05" sheetId="6" r:id="rId2"/>
     <sheet name="05-05" sheetId="7" r:id="rId3"/>
     <sheet name="06-05" sheetId="8" r:id="rId4"/>
+    <sheet name="07-05" sheetId="9" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1702" uniqueCount="627">
   <si>
     <t>THU 6</t>
   </si>
@@ -1352,33 +1353,51 @@
     <t>KIM LIÊN</t>
   </si>
   <si>
+    <t>25/17/11 CỬU LONG PHƯỜNG 2</t>
+  </si>
+  <si>
     <t>06-05-2026</t>
   </si>
   <si>
+    <t>Su Anh</t>
+  </si>
+  <si>
+    <t>22/40 Yên Thế, P2</t>
+  </si>
+  <si>
     <t>TEQUILA THAO VY</t>
   </si>
   <si>
+    <t>426 nơ trang long</t>
+  </si>
+  <si>
+    <t>TOM AG</t>
+  </si>
+  <si>
+    <t>12 HỒ VĂN HUÊ PHƯỜNG 9</t>
+  </si>
+  <si>
+    <t>Tường Vi</t>
+  </si>
+  <si>
+    <t>HD018651</t>
+  </si>
+  <si>
+    <t>325 phan xích long</t>
+  </si>
+  <si>
+    <t>C Phước - fb Yến Nguyễn</t>
+  </si>
+  <si>
+    <t>HD018741</t>
+  </si>
+  <si>
+    <t>Block C 685 Âu Cơ, Chung Cư Oriental Plaza</t>
+  </si>
+  <si>
     <t>AT 06-05</t>
   </si>
   <si>
-    <t>Tường Vi</t>
-  </si>
-  <si>
-    <t>HD018651</t>
-  </si>
-  <si>
-    <t>325 phan xích long</t>
-  </si>
-  <si>
-    <t>C Phước - fb Yến Nguyễn</t>
-  </si>
-  <si>
-    <t>HD018741</t>
-  </si>
-  <si>
-    <t>Block C 685 Âu Cơ, Chung Cư Oriental Plaza</t>
-  </si>
-  <si>
     <t>Phạm Vui</t>
   </si>
   <si>
@@ -1394,6 +1413,9 @@
     <t>HD018829</t>
   </si>
   <si>
+    <t>68A trung mỹ tây 3, phường trung mỹ tây</t>
+  </si>
+  <si>
     <t>Tâm Như</t>
   </si>
   <si>
@@ -1409,12 +1431,18 @@
     <t>HD018739</t>
   </si>
   <si>
+    <t>41a phú định p16</t>
+  </si>
+  <si>
     <t>Trúc Ly</t>
   </si>
   <si>
     <t>HD018824</t>
   </si>
   <si>
+    <t>280 Bình Trị Đông, Phường Bình Trị Đông</t>
+  </si>
+  <si>
     <t>Fb: Vân Nhung</t>
   </si>
   <si>
@@ -1430,12 +1458,18 @@
     <t>HD018784</t>
   </si>
   <si>
+    <t>21/41 bình lợi p13</t>
+  </si>
+  <si>
     <t>Jasploy9989 (inst slideincloset)</t>
   </si>
   <si>
     <t>HD018695</t>
   </si>
   <si>
+    <t>275/14B1 Đặng Nguyên Cẩn, Phường Phú Lâm (phường 14 cũ)</t>
+  </si>
+  <si>
     <t>Lê Thảo</t>
   </si>
   <si>
@@ -1451,6 +1485,9 @@
     <t>HD018652</t>
   </si>
   <si>
+    <t>Chung cư Sai Gon Avenue - Đường số 11, khu phố 4, phường Tam Bình</t>
+  </si>
+  <si>
     <t>Ánh Tuyết</t>
   </si>
   <si>
@@ -1460,15 +1497,36 @@
     <t>23 lộc hưng p6</t>
   </si>
   <si>
+    <t>Hoàng Thúy Triều</t>
+  </si>
+  <si>
+    <t>HD018807</t>
+  </si>
+  <si>
+    <t>477 19 nguyễn văn công p3</t>
+  </si>
+  <si>
+    <t>Michelle Nguyen (Tu Anh)</t>
+  </si>
+  <si>
     <t>HD018799</t>
   </si>
   <si>
+    <t>19 Yên Thế p.2</t>
+  </si>
+  <si>
     <t>Charii ( inst chari_importshop )-BN2441</t>
   </si>
   <si>
     <t>HD018456</t>
   </si>
   <si>
+    <t>163 Trương Thị Hoa, phường Tân Thới Hiệp</t>
+  </si>
+  <si>
+    <t>Tên dinh - fb NG Eric 0đ</t>
+  </si>
+  <si>
     <t>HD018721</t>
   </si>
   <si>
@@ -1481,60 +1539,90 @@
     <t>HD018610</t>
   </si>
   <si>
+    <t>8 đường 19 phường Bình Trị Đông B</t>
+  </si>
+  <si>
     <t>Gia Linh</t>
   </si>
   <si>
     <t>HD018601</t>
   </si>
   <si>
+    <t>100 đinh văn ước ấp5 xã hưng long</t>
+  </si>
+  <si>
     <t>Thiên Trang</t>
   </si>
   <si>
     <t>HD018668</t>
   </si>
   <si>
+    <t>221 trần bình trọng p2</t>
+  </si>
+  <si>
     <t>Nam Diep Hung Tue</t>
   </si>
   <si>
     <t>HD018802</t>
   </si>
   <si>
+    <t>Chung cư Sơn Kỳ 2 số 37 đường DC 13 p Tây Thạnh</t>
+  </si>
+  <si>
     <t>BN182 miki chouchou Fb</t>
   </si>
   <si>
     <t>HD018603</t>
   </si>
   <si>
+    <t>163 Đường Trương Thị Hoa, phường Tân Thới Hiệp</t>
+  </si>
+  <si>
     <t>Phượng Nhi</t>
   </si>
   <si>
     <t>HD018622</t>
   </si>
   <si>
+    <t>35 đặng thị nhu phường Nguyễn thái bình</t>
+  </si>
+  <si>
     <t>Lý Ngọc Khuyên ( 1805) fb Jessy Dang</t>
   </si>
   <si>
     <t>HD018774</t>
   </si>
   <si>
+    <t>Toà nhà Bảy Hiền : 9 Phạm Phu Thử, nay phường Bảy Hiền (phuong 11 cũ)</t>
+  </si>
+  <si>
     <t>Quỳnh Hương</t>
   </si>
   <si>
     <t>HD018593</t>
   </si>
   <si>
+    <t>Saigon Royal Residence, Nguyễn Trường Tộ, phường 13</t>
+  </si>
+  <si>
     <t>Huỳnh Thị Thúy Kiều</t>
   </si>
   <si>
     <t>HD018671</t>
   </si>
   <si>
+    <t>Chung cư zentower 34/1 ql1 phường thới an</t>
+  </si>
+  <si>
     <t>Macie Nguyen</t>
   </si>
   <si>
     <t>HD018621</t>
   </si>
   <si>
+    <t>91 Phạm Văn Hai, f3</t>
+  </si>
+  <si>
     <t>Trân Hoàng Kỳ Châu</t>
   </si>
   <si>
@@ -1544,91 +1632,295 @@
     <t>Công ty TNHH GỐM sứ Kim Trúc, khu công nghiệp Tân Bình, đường số 3 lô 4, phường Tây Thạnh</t>
   </si>
   <si>
-    <t>25/17/11 CỬU LONG PHƯỜNG 2</t>
-  </si>
-  <si>
-    <t>22/40 Yên Thế, P2</t>
-  </si>
-  <si>
-    <t>426 nơ trang long</t>
-  </si>
-  <si>
-    <t>163 Trương Thị Hoa, phường Tân Thới Hiệp</t>
-  </si>
-  <si>
-    <t>21/41 bình lợi p13</t>
-  </si>
-  <si>
-    <t>Hoàng Thúy Triều</t>
-  </si>
-  <si>
-    <t>HD018807</t>
-  </si>
-  <si>
-    <t>477 19 nguyễn văn công p3</t>
-  </si>
-  <si>
-    <t>163 Đường Trương Thị Hoa, phường Tân Thới Hiệp</t>
-  </si>
-  <si>
-    <t>Chung cư Sai Gon Avenue - Đường số 11, khu phố 4, phường Tam Bình</t>
-  </si>
-  <si>
-    <t>12 HỒ VĂN HUÊ PHƯỜNG 9</t>
-  </si>
-  <si>
-    <t>TOM AG</t>
-  </si>
-  <si>
-    <t>Su Anh</t>
-  </si>
-  <si>
-    <t>35 đặng thị nhu phường Nguyễn thái bình</t>
-  </si>
-  <si>
-    <t>Michelle Nguyen (Tu Anh)</t>
-  </si>
-  <si>
-    <t>19 Yên Thế p.2</t>
-  </si>
-  <si>
-    <t>91 Phạm Văn Hai, f3</t>
-  </si>
-  <si>
-    <t>Saigon Royal Residence, Nguyễn Trường Tộ, phường 13</t>
-  </si>
-  <si>
-    <t>221 trần bình trọng p2</t>
-  </si>
-  <si>
-    <t>Chung cư zentower 34/1 ql1 phường thới an</t>
-  </si>
-  <si>
-    <t>100 đinh văn ước ấp5 xã hưng long</t>
-  </si>
-  <si>
-    <t>Tên dinh - fb NG Eric 0đ</t>
-  </si>
-  <si>
-    <t>41a phú định p16</t>
-  </si>
-  <si>
-    <t>Chung cư Sơn Kỳ 2 số 37 đường DC 13 p Tây Thạnh</t>
-  </si>
-  <si>
-    <t>280 Bình Trị Đông, Phường Bình Trị Đông</t>
-  </si>
-  <si>
-    <t>8 đường 19 phường Bình Trị Đông B</t>
-  </si>
-  <si>
-    <t>68A trung mỹ tây 3, phường trung mỹ tây</t>
-  </si>
-  <si>
-    <t>275/14B1 Đặng Nguyên Cẩn, Phường Phú Lâm (phường 14 cũ)</t>
-  </si>
-  <si>
-    <t>Toà nhà Bảy Hiền : 9 Phạm Phu Thử, nay phường Bảy Hiền (phuong 11 cũ)</t>
+    <t>THU 5</t>
+  </si>
+  <si>
+    <t>NGAY 7-5</t>
+  </si>
+  <si>
+    <t>Tuyến fb Có Đuôi Gà</t>
+  </si>
+  <si>
+    <t>HD019062</t>
+  </si>
+  <si>
+    <t>AT 07-05</t>
+  </si>
+  <si>
+    <t>07-05-2026</t>
+  </si>
+  <si>
+    <t>Lê Thị Quỳnh Yến</t>
+  </si>
+  <si>
+    <t>HD019032</t>
+  </si>
+  <si>
+    <t>82 bạch vân</t>
+  </si>
+  <si>
+    <t>Thuỳ Duyên - fb Elyna Tran</t>
+  </si>
+  <si>
+    <t>HD019033</t>
+  </si>
+  <si>
+    <t>Vinhome Grandpark Be3, Nguyễn Xiển, Long Bình</t>
+  </si>
+  <si>
+    <t>Thỏ Selina</t>
+  </si>
+  <si>
+    <t>HD019055</t>
+  </si>
+  <si>
+    <t>HD018836</t>
+  </si>
+  <si>
+    <t>Phương Thảo</t>
+  </si>
+  <si>
+    <t>Huyền</t>
+  </si>
+  <si>
+    <t>HD018987</t>
+  </si>
+  <si>
+    <t>218/10 nam kì khởi nghĩa</t>
+  </si>
+  <si>
+    <t>Phương Phạm</t>
+  </si>
+  <si>
+    <t>HD018958</t>
+  </si>
+  <si>
+    <t>Bs16A vinhome grand park long bình</t>
+  </si>
+  <si>
+    <t>Trang Lê</t>
+  </si>
+  <si>
+    <t>HD019057</t>
+  </si>
+  <si>
+    <t>Lê Thị Minh Phượng.</t>
+  </si>
+  <si>
+    <t>HD019071</t>
+  </si>
+  <si>
+    <t>155/14 ds 11 bình hưng hoà</t>
+  </si>
+  <si>
+    <t>Phạm Thị Bảo Trân</t>
+  </si>
+  <si>
+    <t>HD018909</t>
+  </si>
+  <si>
+    <t>My Nhung Ly</t>
+  </si>
+  <si>
+    <t>HD019061</t>
+  </si>
+  <si>
+    <t>số 13 đường số 9, P13</t>
+  </si>
+  <si>
+    <t>Chị Phương</t>
+  </si>
+  <si>
+    <t>HD019053</t>
+  </si>
+  <si>
+    <t>984/62 hà huy giáp</t>
+  </si>
+  <si>
+    <t>Nguyễn Kim Dung</t>
+  </si>
+  <si>
+    <t>HD019069</t>
+  </si>
+  <si>
+    <t>40/20 trần văn quang p10</t>
+  </si>
+  <si>
+    <t>Thụy Uyên Vũ</t>
+  </si>
+  <si>
+    <t>HD018911</t>
+  </si>
+  <si>
+    <t>Chung cư the manor 2</t>
+  </si>
+  <si>
+    <t>huyền nguyễn</t>
+  </si>
+  <si>
+    <t>HD016429</t>
+  </si>
+  <si>
+    <t>Thu Phương</t>
+  </si>
+  <si>
+    <t>HD018907</t>
+  </si>
+  <si>
+    <t>Uyên Phương ( Trân)</t>
+  </si>
+  <si>
+    <t>HD018834</t>
+  </si>
+  <si>
+    <t>31 Nguyễn Văn Linh, phường Tân Thuận Tây</t>
+  </si>
+  <si>
+    <t>Trần Phương Quỳnh</t>
+  </si>
+  <si>
+    <t>HD018973</t>
+  </si>
+  <si>
+    <t>53 nguyễn thị minh khai, p sài gòn tòa nhà avalon</t>
+  </si>
+  <si>
+    <t>VN ( Allie Biiny)</t>
+  </si>
+  <si>
+    <t>HD018858</t>
+  </si>
+  <si>
+    <t>Kim Hằng</t>
+  </si>
+  <si>
+    <t>HD018939</t>
+  </si>
+  <si>
+    <t>HD018855</t>
+  </si>
+  <si>
+    <t>Phương Thúy</t>
+  </si>
+  <si>
+    <t>HD018990</t>
+  </si>
+  <si>
+    <t>33 đường số 5 cát lái</t>
+  </si>
+  <si>
+    <t>Trần HUỆ</t>
+  </si>
+  <si>
+    <t>HD018874</t>
+  </si>
+  <si>
+    <t>391 ngô gia tự p2</t>
+  </si>
+  <si>
+    <t>HD019025</t>
+  </si>
+  <si>
+    <t>Nguyễn Trang</t>
+  </si>
+  <si>
+    <t>HD018885</t>
+  </si>
+  <si>
+    <t>Diễm Quỳnh</t>
+  </si>
+  <si>
+    <t>HD019054</t>
+  </si>
+  <si>
+    <t>Masteri thảo điền tháp t3 Thao dien</t>
+  </si>
+  <si>
+    <t>HD019058</t>
+  </si>
+  <si>
+    <t>120/3/11 Đăng Thùy Trâm, P13 ( CTY GIA HUY EXPRESS )</t>
+  </si>
+  <si>
+    <t>Ngọc Hân Nghiêm</t>
+  </si>
+  <si>
+    <t>HD018899</t>
+  </si>
+  <si>
+    <t>HD018512</t>
+  </si>
+  <si>
+    <t>CUS TWO EIGHT EIGHT TWO NINE</t>
+  </si>
+  <si>
+    <t>HD018877</t>
+  </si>
+  <si>
+    <t>270B LÝ THƯỜNG KIỆT KP1 P6</t>
+  </si>
+  <si>
+    <t>Thanh Thanh Trương</t>
+  </si>
+  <si>
+    <t>HD019041</t>
+  </si>
+  <si>
+    <t>518/24 võ văn kiệt</t>
+  </si>
+  <si>
+    <t>7/88, Ik 5-6, bình Hưng hoà B</t>
+  </si>
+  <si>
+    <t>124 đường số 9 KDC Bình Hưng, Bình Hưng</t>
+  </si>
+  <si>
+    <t>chung cư the park residence. 12 nguyễn hữu thọ phước kien</t>
+  </si>
+  <si>
+    <t>Phương 1 Street/Buildding Name: \450/28Gdương bá trạc(061771181)</t>
+  </si>
+  <si>
+    <t>96a đg 79 phường tân quy</t>
+  </si>
+  <si>
+    <t>PARK VIEW APARTMENT R4-10-11, Hưng Gia 1,Đ. Số 2, Tân Phong</t>
+  </si>
+  <si>
+    <t>ái quyên mai malaysia</t>
+  </si>
+  <si>
+    <t>22 Tân Thới Nhất 1B, p. Tân Thới Nhất</t>
+  </si>
+  <si>
+    <t>8A Sông Thương P2</t>
+  </si>
+  <si>
+    <t>Chung cư freshca lock b Phường Bình Chiểu</t>
+  </si>
+  <si>
+    <t>Tháp S2 - The sun avenue 28 Mai Chí Thọ, P bình trưng</t>
+  </si>
+  <si>
+    <t>ELLY NGUYỄN - THẮM NGUYÊN</t>
+  </si>
+  <si>
+    <t>Block B Chung Cư Urban Green, Đường Số 6, Hiệp Bình</t>
+  </si>
+  <si>
+    <t>HD018831</t>
+  </si>
+  <si>
+    <t>504 Nguyễn Tất Thành, phường 18 chung cư Riva Park</t>
+  </si>
+  <si>
+    <t>HD018959</t>
+  </si>
+  <si>
+    <t>hải my fb Bé Hân</t>
+  </si>
+  <si>
+    <t>31 an bình P6</t>
   </si>
 </sst>
 </file>
@@ -7079,9 +7371,1254 @@
   <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="36.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="114.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0</v>
+      </c>
+      <c r="H3" s="6">
+        <v>30</v>
+      </c>
+      <c r="I3" s="6">
+        <f t="shared" ref="I3:I34" si="0">G3-H3</f>
+        <v>-30</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>30</v>
+      </c>
+      <c r="I4" s="6">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3">
+        <v>25</v>
+      </c>
+      <c r="I5" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="G6" s="6">
+        <v>25</v>
+      </c>
+      <c r="H6" s="6">
+        <v>25</v>
+      </c>
+      <c r="I6" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="G7" s="6">
+        <v>4860</v>
+      </c>
+      <c r="H7" s="6">
+        <v>30</v>
+      </c>
+      <c r="I7" s="6">
+        <f t="shared" si="0"/>
+        <v>4830</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>450</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8">
+        <v>25</v>
+      </c>
+      <c r="I8" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G9" s="3">
+        <v>985</v>
+      </c>
+      <c r="H9" s="3">
+        <v>25</v>
+      </c>
+      <c r="I9" s="3">
+        <f t="shared" si="0"/>
+        <v>960</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>455</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>456</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>457</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="8">
+        <v>400</v>
+      </c>
+      <c r="H10" s="8">
+        <v>30</v>
+      </c>
+      <c r="I10" s="8">
+        <f t="shared" si="0"/>
+        <v>370</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="3">
+        <v>560</v>
+      </c>
+      <c r="H11" s="3">
+        <v>30</v>
+      </c>
+      <c r="I11" s="3">
+        <f t="shared" si="0"/>
+        <v>530</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="8">
+        <v>1060</v>
+      </c>
+      <c r="H12" s="8">
+        <v>30</v>
+      </c>
+      <c r="I12" s="8">
+        <f t="shared" si="0"/>
+        <v>1030</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="8">
+        <v>820</v>
+      </c>
+      <c r="H13" s="8">
+        <v>30</v>
+      </c>
+      <c r="I13" s="8">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" s="3">
+        <v>815</v>
+      </c>
+      <c r="H14" s="3">
+        <v>25</v>
+      </c>
+      <c r="I14" s="3">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G15" s="3">
+        <v>1140</v>
+      </c>
+      <c r="H15" s="3">
+        <v>20</v>
+      </c>
+      <c r="I15" s="3">
+        <f t="shared" si="0"/>
+        <v>1120</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>473</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>474</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="G16" s="8">
+        <v>0</v>
+      </c>
+      <c r="H16" s="8">
+        <v>25</v>
+      </c>
+      <c r="I16" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="6">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6">
+        <v>25</v>
+      </c>
+      <c r="I17" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="3">
+        <v>410</v>
+      </c>
+      <c r="H18" s="3">
+        <v>30</v>
+      </c>
+      <c r="I18" s="3">
+        <f t="shared" si="0"/>
+        <v>380</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" s="6">
+        <v>795</v>
+      </c>
+      <c r="H19" s="6">
+        <v>25</v>
+      </c>
+      <c r="I19" s="6">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3">
+        <v>25</v>
+      </c>
+      <c r="I20" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="6">
+        <v>0</v>
+      </c>
+      <c r="H21" s="6">
+        <v>25</v>
+      </c>
+      <c r="I21" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3">
+        <v>30</v>
+      </c>
+      <c r="I22" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>495</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>496</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G23" s="8">
+        <v>890</v>
+      </c>
+      <c r="H23" s="8">
+        <v>30</v>
+      </c>
+      <c r="I23" s="8">
+        <f t="shared" si="0"/>
+        <v>860</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>497</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="8">
+        <v>850</v>
+      </c>
+      <c r="H24" s="8">
+        <v>30</v>
+      </c>
+      <c r="I24" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" s="8">
+        <v>855</v>
+      </c>
+      <c r="H25" s="8">
+        <v>35</v>
+      </c>
+      <c r="I25" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G26" s="6">
+        <v>25</v>
+      </c>
+      <c r="H26" s="6">
+        <v>25</v>
+      </c>
+      <c r="I26" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="M26" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>507</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>508</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="8">
+        <v>1175</v>
+      </c>
+      <c r="H27" s="8">
+        <v>25</v>
+      </c>
+      <c r="I27" s="8">
+        <f t="shared" si="0"/>
+        <v>1150</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>30</v>
+      </c>
+      <c r="I28" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G29" s="6">
+        <v>1475</v>
+      </c>
+      <c r="H29" s="6">
+        <v>25</v>
+      </c>
+      <c r="I29" s="6">
+        <f t="shared" si="0"/>
+        <v>1450</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>516</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>517</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G30" s="8">
+        <v>715</v>
+      </c>
+      <c r="H30" s="8">
+        <v>25</v>
+      </c>
+      <c r="I30" s="8">
+        <f t="shared" si="0"/>
+        <v>690</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="G31" s="6">
+        <v>825</v>
+      </c>
+      <c r="H31" s="6">
+        <v>25</v>
+      </c>
+      <c r="I31" s="6">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>523</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G32" s="8">
+        <v>1150</v>
+      </c>
+      <c r="H32" s="8">
+        <v>30</v>
+      </c>
+      <c r="I32" s="8">
+        <f t="shared" si="0"/>
+        <v>1120</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G33" s="6">
+        <v>3370</v>
+      </c>
+      <c r="H33" s="6">
+        <v>30</v>
+      </c>
+      <c r="I33" s="6">
+        <f t="shared" si="0"/>
+        <v>3340</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>527</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>529</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G34" s="8">
+        <v>0</v>
+      </c>
+      <c r="H34" s="8">
+        <v>25</v>
+      </c>
+      <c r="I34" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:P36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="77" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -7092,10 +8629,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>434</v>
+        <v>530</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>435</v>
+        <v>531</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -7148,67 +8685,67 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>501</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="G3" s="6">
+    <row r="3" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>533</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="8">
         <v>0</v>
       </c>
-      <c r="H3" s="6">
-        <v>30</v>
-      </c>
-      <c r="I3" s="6">
-        <f t="shared" ref="I3:I34" si="0">G3-H3</f>
+      <c r="H3" s="8">
+        <v>30</v>
+      </c>
+      <c r="I3" s="8">
+        <f t="shared" ref="I3:I36" si="0">G3-H3</f>
         <v>-30</v>
       </c>
-      <c r="J3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>437</v>
+      <c r="J3" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>193</v>
-      </c>
       <c r="B4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>513</v>
+        <v>536</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>537</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>502</v>
+        <v>538</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="G4" s="6">
-        <v>0</v>
+        <v>1175</v>
       </c>
       <c r="H4" s="6">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I4" s="6">
         <f t="shared" si="0"/>
-        <v>-30</v>
+        <v>1150</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>37</v>
@@ -7217,229 +8754,223 @@
         <v>24</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>438</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G5" s="3">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>539</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G5" s="5">
+        <v>850</v>
+      </c>
+      <c r="H5" s="5">
+        <v>30</v>
+      </c>
+      <c r="I5" s="5">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="3">
+        <v>850</v>
+      </c>
+      <c r="H6" s="3">
+        <v>30</v>
+      </c>
+      <c r="I6" s="3">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="3">
         <v>0</v>
       </c>
-      <c r="H5" s="3">
-        <v>25</v>
-      </c>
-      <c r="I5" s="3">
+      <c r="H7" s="3">
+        <v>30</v>
+      </c>
+      <c r="I7" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="G8" s="6">
+        <v>765</v>
+      </c>
+      <c r="H8" s="6">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6">
+        <f t="shared" si="0"/>
+        <v>740</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>25</v>
+      </c>
+      <c r="I9" s="6">
         <f t="shared" si="0"/>
         <v>-25</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>437</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>512</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>355</v>
-      </c>
-      <c r="G6" s="6">
-        <v>25</v>
-      </c>
-      <c r="H6" s="6">
-        <v>25</v>
-      </c>
-      <c r="I6" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J6" s="6" t="s">
+      <c r="J9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>441</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>442</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>355</v>
-      </c>
-      <c r="G7" s="6">
-        <v>4860</v>
-      </c>
-      <c r="H7" s="6">
-        <v>30</v>
-      </c>
-      <c r="I7" s="6">
-        <f t="shared" si="0"/>
-        <v>4830</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>443</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>444</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>445</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G8" s="8">
-        <v>0</v>
-      </c>
-      <c r="H8" s="8">
-        <v>25</v>
-      </c>
-      <c r="I8" s="8">
-        <f t="shared" si="0"/>
-        <v>-25</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>446</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>447</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>448</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G9" s="3">
-        <v>985</v>
-      </c>
-      <c r="H9" s="3">
-        <v>25</v>
-      </c>
-      <c r="I9" s="3">
-        <f t="shared" si="0"/>
-        <v>960</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>449</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>450</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>527</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="8">
-        <v>400</v>
-      </c>
-      <c r="H10" s="8">
-        <v>30</v>
-      </c>
-      <c r="I10" s="8">
-        <f t="shared" si="0"/>
-        <v>370</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>437</v>
+      <c r="K9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" s="5">
+        <v>750</v>
+      </c>
+      <c r="H10" s="5">
+        <v>30</v>
+      </c>
+      <c r="I10" s="5">
+        <f t="shared" si="0"/>
+        <v>720</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7447,26 +8978,26 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>451</v>
+        <v>552</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>452</v>
+        <v>553</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>453</v>
+        <v>617</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="G11" s="3">
-        <v>560</v>
+        <v>2200</v>
       </c>
       <c r="H11" s="3">
         <v>30</v>
       </c>
       <c r="I11" s="3">
         <f t="shared" si="0"/>
-        <v>530</v>
+        <v>2170</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>24</v>
@@ -7475,7 +9006,10 @@
         <v>24</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>437</v>
+        <v>535</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -7483,143 +9017,143 @@
         <v>18</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>454</v>
+        <v>554</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>455</v>
+        <v>555</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>523</v>
+        <v>556</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="G12" s="8">
-        <v>1060</v>
+        <v>900</v>
       </c>
       <c r="H12" s="8">
         <v>30</v>
       </c>
       <c r="I12" s="8">
         <f t="shared" si="0"/>
-        <v>1030</v>
+        <v>870</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>439</v>
+        <v>534</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>456</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>457</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>525</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="G13" s="8">
-        <v>820</v>
-      </c>
-      <c r="H13" s="8">
-        <v>30</v>
-      </c>
-      <c r="I13" s="8">
-        <f t="shared" si="0"/>
-        <v>790</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G14" s="3">
-        <v>815</v>
-      </c>
-      <c r="H14" s="3">
-        <v>25</v>
-      </c>
-      <c r="I14" s="3">
-        <f t="shared" si="0"/>
-        <v>790</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>462</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>505</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G15" s="3">
-        <v>1140</v>
-      </c>
-      <c r="H15" s="3">
-        <v>20</v>
-      </c>
-      <c r="I15" s="3">
-        <f t="shared" si="0"/>
-        <v>1120</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>437</v>
+        <v>535</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="3">
+        <v>670</v>
+      </c>
+      <c r="H13" s="3">
+        <v>30</v>
+      </c>
+      <c r="I13" s="3">
+        <f t="shared" si="0"/>
+        <v>640</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>561</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="G14" s="8">
+        <v>775</v>
+      </c>
+      <c r="H14" s="8">
+        <v>25</v>
+      </c>
+      <c r="I14" s="8">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>563</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>564</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="8">
+        <v>400</v>
+      </c>
+      <c r="H15" s="8">
+        <v>30</v>
+      </c>
+      <c r="I15" s="8">
+        <f t="shared" si="0"/>
+        <v>370</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -7627,16 +9161,16 @@
         <v>18</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>463</v>
+        <v>565</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>464</v>
+        <v>566</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>528</v>
+        <v>567</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="G16" s="8">
         <v>0</v>
@@ -7649,229 +9183,229 @@
         <v>-25</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>439</v>
+        <v>534</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>465</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="F17" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3">
+        <v>20</v>
+      </c>
+      <c r="I17" s="3">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" s="6">
+        <v>685</v>
+      </c>
+      <c r="H18" s="6">
+        <v>25</v>
+      </c>
+      <c r="I18" s="6">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>573</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>613</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G19" s="8">
+        <v>850</v>
+      </c>
+      <c r="H19" s="8">
+        <v>30</v>
+      </c>
+      <c r="I19" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G20" s="8">
+        <v>480</v>
+      </c>
+      <c r="H20" s="8">
+        <v>30</v>
+      </c>
+      <c r="I20" s="8">
+        <f t="shared" si="0"/>
+        <v>450</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>579</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="F21" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G21" s="8">
+        <v>1135</v>
+      </c>
+      <c r="H21" s="8">
+        <v>25</v>
+      </c>
+      <c r="I21" s="8">
+        <f t="shared" si="0"/>
+        <v>1110</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>582</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>612</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G22" s="8">
         <v>0</v>
       </c>
-      <c r="H17" s="6">
-        <v>25</v>
-      </c>
-      <c r="I17" s="6">
-        <f t="shared" si="0"/>
-        <v>-25</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L17" s="6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>469</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>510</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G18" s="3">
-        <v>410</v>
-      </c>
-      <c r="H18" s="3">
-        <v>30</v>
-      </c>
-      <c r="I18" s="3">
-        <f t="shared" si="0"/>
-        <v>380</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>470</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>471</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>472</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="G19" s="6">
-        <v>795</v>
-      </c>
-      <c r="H19" s="6">
-        <v>25</v>
-      </c>
-      <c r="I19" s="6">
-        <f t="shared" si="0"/>
-        <v>770</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L19" s="6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="20" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>508</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G20" s="3">
-        <v>0</v>
-      </c>
-      <c r="H20" s="3">
-        <v>25</v>
-      </c>
-      <c r="I20" s="3">
-        <f t="shared" si="0"/>
-        <v>-25</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="21" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>515</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>473</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="G21" s="6">
-        <v>0</v>
-      </c>
-      <c r="H21" s="6">
-        <v>25</v>
-      </c>
-      <c r="I21" s="6">
-        <f t="shared" si="0"/>
-        <v>-25</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="22" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>504</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G22" s="3">
-        <v>0</v>
-      </c>
-      <c r="H22" s="3">
-        <v>30</v>
-      </c>
-      <c r="I22" s="3">
+      <c r="H22" s="8">
+        <v>30</v>
+      </c>
+      <c r="I22" s="8">
         <f t="shared" si="0"/>
         <v>-30</v>
       </c>
-      <c r="J22" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>437</v>
+      <c r="J22" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="23" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -7879,35 +9413,35 @@
         <v>18</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>522</v>
+        <v>583</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>476</v>
+        <v>584</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>477</v>
+        <v>614</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>22</v>
+        <v>131</v>
       </c>
       <c r="G23" s="8">
-        <v>890</v>
+        <v>670</v>
       </c>
       <c r="H23" s="8">
         <v>30</v>
       </c>
       <c r="I23" s="8">
         <f t="shared" si="0"/>
-        <v>860</v>
+        <v>640</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>439</v>
+        <v>534</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L23" s="8" t="s">
-        <v>437</v>
+        <v>535</v>
       </c>
     </row>
     <row r="24" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -7915,71 +9449,74 @@
         <v>18</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>478</v>
+        <v>33</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>479</v>
+        <v>585</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>526</v>
+        <v>611</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="G24" s="8">
-        <v>850</v>
+        <v>95</v>
       </c>
       <c r="H24" s="8">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="I24" s="8">
         <f t="shared" si="0"/>
-        <v>820</v>
+        <v>60</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>439</v>
+        <v>534</v>
       </c>
       <c r="K24" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="25" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>480</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>481</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>521</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="G25" s="8">
-        <v>855</v>
-      </c>
-      <c r="H25" s="8">
-        <v>35</v>
-      </c>
-      <c r="I25" s="8">
-        <f t="shared" si="0"/>
-        <v>820</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>437</v>
+        <v>535</v>
+      </c>
+      <c r="M24" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>586</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" s="3">
+        <v>690</v>
+      </c>
+      <c r="H25" s="3">
+        <v>30</v>
+      </c>
+      <c r="I25" s="3">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="26" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -7987,26 +9524,26 @@
         <v>18</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>482</v>
+        <v>589</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>483</v>
+        <v>590</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>519</v>
+        <v>591</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>59</v>
+        <v>308</v>
       </c>
       <c r="G26" s="6">
-        <v>25</v>
+        <v>865</v>
       </c>
       <c r="H26" s="6">
         <v>25</v>
       </c>
       <c r="I26" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>840</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>37</v>
@@ -8015,46 +9552,46 @@
         <v>24</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="M26" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G27" s="3">
+        <v>30</v>
+      </c>
+      <c r="H27" s="3">
+        <v>30</v>
+      </c>
+      <c r="I27" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="M27" s="3" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="27" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>484</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>485</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>524</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G27" s="8">
-        <v>1175</v>
-      </c>
-      <c r="H27" s="8">
-        <v>25</v>
-      </c>
-      <c r="I27" s="8">
-        <f t="shared" si="0"/>
-        <v>1150</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K27" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="28" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8062,143 +9599,146 @@
         <v>18</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>486</v>
+        <v>593</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>487</v>
+        <v>594</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>509</v>
+        <v>618</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="G28" s="3">
+        <v>780</v>
+      </c>
+      <c r="H28" s="3">
+        <v>30</v>
+      </c>
+      <c r="I28" s="3">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G29" s="3">
+        <v>850</v>
+      </c>
+      <c r="H29" s="3">
+        <v>30</v>
+      </c>
+      <c r="I29" s="3">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G30" s="3">
         <v>0</v>
       </c>
-      <c r="H28" s="3">
-        <v>30</v>
-      </c>
-      <c r="I28" s="3">
-        <f t="shared" si="0"/>
-        <v>-30</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="29" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>488</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="G29" s="6">
-        <v>1475</v>
-      </c>
-      <c r="H29" s="6">
-        <v>25</v>
-      </c>
-      <c r="I29" s="6">
-        <f t="shared" si="0"/>
-        <v>1450</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="30" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>490</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>491</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>529</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="G30" s="8">
-        <v>715</v>
-      </c>
-      <c r="H30" s="8">
-        <v>25</v>
-      </c>
-      <c r="I30" s="8">
-        <f t="shared" si="0"/>
-        <v>690</v>
-      </c>
-      <c r="J30" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K30" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L30" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="31" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>518</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="G31" s="6">
-        <v>825</v>
-      </c>
-      <c r="H31" s="6">
-        <v>25</v>
-      </c>
-      <c r="I31" s="6">
-        <f t="shared" si="0"/>
-        <v>800</v>
-      </c>
-      <c r="J31" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K31" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L31" s="6" t="s">
-        <v>437</v>
+      <c r="H30" s="3">
+        <v>20</v>
+      </c>
+      <c r="I30" s="3">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>600</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>601</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>610</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G31" s="8">
+        <v>0</v>
+      </c>
+      <c r="H31" s="8">
+        <v>35</v>
+      </c>
+      <c r="I31" s="8">
+        <f t="shared" ref="I31" si="1">G31-H31</f>
+        <v>-35</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="M31" s="8" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="32" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -8206,62 +9746,65 @@
         <v>18</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>494</v>
+        <v>600</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>495</v>
+        <v>602</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>520</v>
+        <v>610</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="G32" s="8">
-        <v>1150</v>
+        <v>0</v>
       </c>
       <c r="H32" s="8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I32" s="8">
         <f t="shared" si="0"/>
-        <v>1120</v>
+        <v>0</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>439</v>
+        <v>534</v>
       </c>
       <c r="K32" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L32" s="8" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="33" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+        <v>535</v>
+      </c>
+      <c r="M32" s="8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>496</v>
+        <v>603</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>497</v>
+        <v>604</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>517</v>
+        <v>605</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>102</v>
       </c>
       <c r="G33" s="6">
-        <v>3370</v>
+        <v>0</v>
       </c>
       <c r="H33" s="6">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I33" s="6">
         <f t="shared" si="0"/>
-        <v>3340</v>
+        <v>-25</v>
       </c>
       <c r="J33" s="6" t="s">
         <v>37</v>
@@ -8270,49 +9813,122 @@
         <v>24</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="M33" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G34" s="6">
+        <v>0</v>
+      </c>
+      <c r="H34" s="6">
+        <v>25</v>
+      </c>
+      <c r="I34" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G35" s="6">
+        <v>2050</v>
+      </c>
+      <c r="H35" s="6">
+        <v>30</v>
+      </c>
+      <c r="I35" s="6">
+        <f t="shared" si="0"/>
+        <v>2020</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="M35" s="6" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="34" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>498</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>499</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>500</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G34" s="8">
+    <row r="36" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G36" s="3">
+        <v>30</v>
+      </c>
+      <c r="H36" s="3">
+        <v>30</v>
+      </c>
+      <c r="I36" s="3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="8">
-        <v>25</v>
-      </c>
-      <c r="I34" s="8">
-        <f t="shared" si="0"/>
-        <v>-25</v>
-      </c>
-      <c r="J34" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="K34" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L34" s="8" t="s">
-        <v>437</v>
+      <c r="J36" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>535</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>